<commit_message>
Refine extra experiments, tune case 2, and update control figures
</commit_message>
<xml_diff>
--- a/extra_experiment/results/extra_experiment_summary.xlsx
+++ b/extra_experiment/results/extra_experiment_summary.xlsx
@@ -535,28 +535,28 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2.183607723991278</v>
+        <v>0.3905449124521958</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0001872310686431242</v>
+        <v>0.0001000002942015</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01717636639409803</v>
+        <v>0.0216305229189037</v>
       </c>
       <c r="D2" t="n">
-        <v>5.245771695576813</v>
+        <v>0.0010000014989995</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4948016203346482</v>
+        <v>1.034905513767046</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7661034226379607</v>
+        <v>29.99999980889567</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0001180574053177272</v>
+        <v>29.99985380292416</v>
       </c>
       <c r="H2" t="n">
-        <v>29.78316639294983</v>
+        <v>3.434922869669779</v>
       </c>
       <c r="I2" t="n">
         <v>120</v>
@@ -565,22 +565,22 @@
         <v>79</v>
       </c>
       <c r="K2" t="n">
-        <v>201</v>
+        <v>29</v>
       </c>
       <c r="L2" t="n">
         <v>7</v>
       </c>
       <c r="M2" t="n">
-        <v>31.89680763352797</v>
+        <v>6.489676808043153</v>
       </c>
       <c r="N2" t="n">
-        <v>22.13463123515775</v>
+        <v>3.992595766657875</v>
       </c>
       <c r="O2" t="n">
-        <v>-0.335996690632808</v>
+        <v>0.9790122976207644</v>
       </c>
       <c r="P2" t="n">
-        <v>49.2817566883381</v>
+        <v>84.65161871886525</v>
       </c>
       <c r="Q2" t="b">
         <v>1</v>
@@ -589,7 +589,7 @@
         <v>2</v>
       </c>
       <c r="S2" t="n">
-        <v>368170.6472686213</v>
+        <v>282042082.4498641</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -599,28 +599,28 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.3978912440618563</v>
+        <v>0.3843465219621007</v>
       </c>
       <c r="B3" t="n">
-        <v>0.7224131431397016</v>
+        <v>0.7177562115288758</v>
       </c>
       <c r="C3" t="n">
-        <v>1.000000001785118e-06</v>
+        <v>1.000000006337894e-06</v>
       </c>
       <c r="D3" t="n">
-        <v>0.001290812504100476</v>
+        <v>0.001586771117871245</v>
       </c>
       <c r="E3" t="n">
-        <v>0.05000000015365245</v>
+        <v>0.05000000000189216</v>
       </c>
       <c r="F3" t="n">
-        <v>20.47790795217968</v>
+        <v>20.52775010233096</v>
       </c>
       <c r="G3" t="n">
-        <v>19.74311798023271</v>
+        <v>16.80191446434893</v>
       </c>
       <c r="H3" t="n">
-        <v>94.18883335159008</v>
+        <v>93.64430412377629</v>
       </c>
       <c r="I3" t="n">
         <v>120</v>
@@ -635,13 +635,13 @@
         <v>7</v>
       </c>
       <c r="M3" t="n">
-        <v>7.229874654036464</v>
+        <v>7.164479595673808</v>
       </c>
       <c r="N3" t="n">
-        <v>5.692474420820583</v>
+        <v>5.761027712292599</v>
       </c>
       <c r="O3" t="n">
-        <v>0.8440103627454674</v>
+        <v>0.8468194894651451</v>
       </c>
       <c r="P3" t="n">
         <v>34.97332316685581</v>
@@ -650,10 +650,10 @@
         <v>1</v>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S3" t="n">
-        <v>130113364.4278214</v>
+        <v>420533309.3137497</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -759,28 +759,28 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7659.715216393337</v>
+        <v>7866.110176160276</v>
       </c>
       <c r="D2" t="n">
-        <v>116.3441240740265</v>
+        <v>152.1781028367666</v>
       </c>
       <c r="E2" t="n">
-        <v>84.48023806553836</v>
+        <v>79</v>
       </c>
       <c r="F2" t="n">
-        <v>147.2287901473712</v>
+        <v>208.9997558863164</v>
       </c>
       <c r="G2" t="n">
-        <v>42.50504720795271</v>
+        <v>19.71246864587363</v>
       </c>
       <c r="H2" t="n">
-        <v>100</v>
+        <v>69.86392989931674</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>30.13607010068326</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -790,7 +790,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>optimizer start 1</t>
+          <t>optimizer start 2</t>
         </is>
       </c>
       <c r="N2" t="b">
@@ -809,38 +809,38 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-2703.982631579588</v>
+        <v>5381.423055594991</v>
       </c>
       <c r="D3" t="n">
-        <v>90.18003433043468</v>
+        <v>140.8720540877382</v>
       </c>
       <c r="E3" t="n">
-        <v>68.76338113697204</v>
+        <v>76.94498209211014</v>
       </c>
       <c r="F3" t="n">
-        <v>107.1675591011654</v>
+        <v>197.5568375134342</v>
       </c>
       <c r="G3" t="n">
-        <v>99.43284323154018</v>
+        <v>20.01992794862599</v>
       </c>
       <c r="H3" t="n">
-        <v>99.43284323154018</v>
+        <v>78.70885892746564</v>
       </c>
       <c r="I3" t="n">
-        <v>0.5671567684598284</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>21.29114107253437</v>
       </c>
       <c r="K3" t="n">
-        <v>27.70629419461152</v>
+        <v>26.87740801847369</v>
       </c>
       <c r="L3" t="n">
-        <v>7.575818078493955</v>
+        <v>10</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>optimizer start 1</t>
+          <t>optimizer start 2</t>
         </is>
       </c>
       <c r="N3" t="b">
@@ -859,25 +859,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-267.9006207090761</v>
+        <v>-335.5106297730085</v>
       </c>
       <c r="D4" t="n">
-        <v>99.59283898372341</v>
+        <v>99.27160283139777</v>
       </c>
       <c r="E4" t="n">
         <v>65</v>
       </c>
       <c r="F4" t="n">
-        <v>122.2185530678835</v>
+        <v>121.0498245699001</v>
       </c>
       <c r="G4" t="n">
-        <v>59.41384264619192</v>
+        <v>62.91079134108784</v>
       </c>
       <c r="H4" t="n">
-        <v>98.10552134302532</v>
+        <v>99.12676375393804</v>
       </c>
       <c r="I4" t="n">
-        <v>1.894478656974693</v>
+        <v>0.8732362460619677</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -890,7 +890,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>optimizer start 1</t>
+          <t>optimizer start 2</t>
         </is>
       </c>
       <c r="N4" t="b">
@@ -909,38 +909,38 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-267.9134345988844</v>
+        <v>-335.5326531668627</v>
       </c>
       <c r="D5" t="n">
-        <v>99.59235481698099</v>
+        <v>99.27075367119713</v>
       </c>
       <c r="E5" t="n">
         <v>65</v>
       </c>
       <c r="F5" t="n">
-        <v>122.2179098845956</v>
+        <v>121.0486961898572</v>
       </c>
       <c r="G5" t="n">
-        <v>59.41491836528826</v>
+        <v>62.91429822010647</v>
       </c>
       <c r="H5" t="n">
-        <v>98.10520201840968</v>
+        <v>99.12668052049385</v>
       </c>
       <c r="I5" t="n">
-        <v>1.894797981590304</v>
+        <v>0.8733194795061567</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1268477373980217</v>
+        <v>0.1675949972364304</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1121794645257455</v>
+        <v>0.146765308101659</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>optimizer start 1</t>
+          <t>optimizer start 2</t>
         </is>
       </c>
       <c r="N5" t="b">
@@ -1005,22 +1005,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-10363.69784797293</v>
+        <v>-2484.687120565285</v>
       </c>
       <c r="C2" t="n">
-        <v>-40.06123104620586</v>
+        <v>-11.44291837288219</v>
       </c>
       <c r="D2" t="n">
-        <v>-15.71685692856632</v>
+        <v>-2.055017907889862</v>
       </c>
       <c r="E2" t="n">
-        <v>56.92779602358746</v>
+        <v>0.3074593027523633</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.5671567684598244</v>
+        <v>8.844929028148897</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5671567684598284</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1030,22 +1030,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.01281388980828524</v>
+        <v>-0.02202339385416963</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.0006431832879343347</v>
+        <v>-0.001128380042842991</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.001075719096334637</v>
+        <v>0.003506879018630116</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0003193246156314444</v>
+        <v>-8.323344418670331e-05</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0003193246156110163</v>
+        <v>8.323344418903478e-05</v>
       </c>
     </row>
   </sheetData>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.109445190650149e-05</v>
+        <v>5.554590669021309e-05</v>
       </c>
     </row>
     <row r="3">
@@ -1106,7 +1106,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.191385156573688e-05</v>
+        <v>5.367754607732422e-05</v>
       </c>
     </row>
     <row r="4">
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.0001129279686580276</v>
+        <v>0.0001133661134247177</v>
       </c>
     </row>
     <row r="5">
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.000112902543193627</v>
+        <v>0.0001134848776018771</v>
       </c>
     </row>
   </sheetData>

</xml_diff>